<commit_message>
Preserve template print layout in generated workbooks
</commit_message>
<xml_diff>
--- a/public/templates/process-docs/厂房支架安装分项工程质量验收表.xlsx
+++ b/public/templates/process-docs/厂房支架安装分项工程质量验收表.xlsx
@@ -1,20 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView windowHeight="17655" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1#厂房" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="第2页" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="1#厂房" sheetId="1" r:id="rId1"/>
+    <sheet name="第2页" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -28,33 +35,31 @@
         <sz val="17"/>
         <color rgb="FF000000"/>
         <rFont val="黑体"/>
-        <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">表</t>
+      <t>表</t>
     </r>
     <r>
       <rPr>
         <sz val="17"/>
         <color rgb="FF000000"/>
         <rFont val="黑体"/>
-        <family val="3"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">5.2 1#</t>
+      <t>5.2 1#</t>
     </r>
     <r>
       <rPr>
         <sz val="17"/>
         <color rgb="FF000000"/>
         <rFont val="黑体"/>
-        <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">厂房支架安装分项工程质量验收表</t>
+      <t>厂房支架安装分项工程质量验收表</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">工程名称：</t>
+    <t>工程名称：</t>
   </si>
   <si>
     <r>
@@ -62,29 +67,27 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">中核汇能高明创楷</t>
+      <t>中核汇能高明创楷</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">3.58904MWP</t>
+      <t>3.58904MWP</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">分布式光伏项目</t>
+      <t>分布式光伏项目</t>
     </r>
   </si>
   <si>
@@ -93,103 +96,102 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">编号：</t>
+      <t>编号：</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
       <t xml:space="preserve">{{文件编号}} </t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">单位（子单位）工程名称</t>
-  </si>
-  <si>
-    <t xml:space="preserve">光伏方阵安装子单位</t>
-  </si>
-  <si>
-    <t xml:space="preserve">分部（子分部）
+    <t>单位（子单位）工程名称</t>
+  </si>
+  <si>
+    <t>光伏方阵安装子单位</t>
+  </si>
+  <si>
+    <t>分部（子分部）
 工程名称</t>
   </si>
   <si>
-    <t xml:space="preserve">子方阵支架及组件安装</t>
-  </si>
-  <si>
-    <t xml:space="preserve">检验批数</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">总承包单位</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{施工单位}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">项目负责人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{施工单位项目负责人}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">项目技术负责人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{总承包单位项目技术负责人}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">施工单位</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{施工单位项目技术负责人}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">分包单位</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{分包单位}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">分包项目负责人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{{分包单位项目负责人}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">分包内容</t>
-  </si>
-  <si>
-    <t xml:space="preserve">工序</t>
-  </si>
-  <si>
-    <t xml:space="preserve">检验项目</t>
-  </si>
-  <si>
-    <t xml:space="preserve">性质</t>
-  </si>
-  <si>
-    <t xml:space="preserve">质量标准</t>
-  </si>
-  <si>
-    <t xml:space="preserve">质量验收结果</t>
-  </si>
-  <si>
-    <t xml:space="preserve">单项
+    <t>子方阵支架及组件安装</t>
+  </si>
+  <si>
+    <t>检验批数</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>总承包单位</t>
+  </si>
+  <si>
+    <t>{{施工单位}}</t>
+  </si>
+  <si>
+    <t>项目负责人</t>
+  </si>
+  <si>
+    <t>{{施工单位项目负责人}}</t>
+  </si>
+  <si>
+    <t>项目技术负责人</t>
+  </si>
+  <si>
+    <t>{{总承包单位项目技术负责人}}</t>
+  </si>
+  <si>
+    <t>施工单位</t>
+  </si>
+  <si>
+    <t>{{施工单位项目技术负责人}}</t>
+  </si>
+  <si>
+    <t>分包单位</t>
+  </si>
+  <si>
+    <t>{{分包单位}}</t>
+  </si>
+  <si>
+    <t>分包项目负责人</t>
+  </si>
+  <si>
+    <t>{{分包单位项目负责人}}</t>
+  </si>
+  <si>
+    <t>分包内容</t>
+  </si>
+  <si>
+    <t>工序</t>
+  </si>
+  <si>
+    <t>检验项目</t>
+  </si>
+  <si>
+    <t>性质</t>
+  </si>
+  <si>
+    <t>质量标准</t>
+  </si>
+  <si>
+    <t>质量验收结果</t>
+  </si>
+  <si>
+    <t>单项
 结论</t>
   </si>
   <si>
-    <t xml:space="preserve">支架安装前准备工作</t>
-  </si>
-  <si>
-    <t xml:space="preserve">现浇混凝土支架基础强度</t>
+    <t>支架安装前准备工作</t>
+  </si>
+  <si>
+    <t>现浇混凝土支架基础强度</t>
   </si>
   <si>
     <r>
@@ -197,19 +199,18 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">混凝土强度达到设计强度的</t>
+      <t>混凝土强度达到设计强度的</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">70%</t>
+      <t>70%</t>
     </r>
   </si>
   <si>
@@ -218,91 +219,88 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">符合</t>
+      <t>符合</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">GB 50171</t>
+      <t>GB 50171</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">中表</t>
+      <t>中表</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">5.0.6</t>
+      <t>5.0.6</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">规定</t>
+      <t>规定</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">支架到场后检查</t>
-  </si>
-  <si>
-    <t xml:space="preserve">外观及防腐涂镀层</t>
-  </si>
-  <si>
-    <t xml:space="preserve">主控</t>
-  </si>
-  <si>
-    <t xml:space="preserve">完好无损</t>
-  </si>
-  <si>
-    <t xml:space="preserve">合格</t>
-  </si>
-  <si>
-    <t xml:space="preserve">型号、规格及材质</t>
-  </si>
-  <si>
-    <t xml:space="preserve">符合设计图纸要求，附件、备件应齐全</t>
-  </si>
-  <si>
-    <t xml:space="preserve">存放在滩涂、盐碱等腐蚀性强的场所的支架</t>
-  </si>
-  <si>
-    <t xml:space="preserve">做好防腐蚀工作</t>
-  </si>
-  <si>
-    <t xml:space="preserve">基础及预埋件（预埋螺栓）的水平偏差和定位轴线偏差</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“中间交接验收签证书”的相关要求</t>
-  </si>
-  <si>
-    <t xml:space="preserve">固定式支架及手动可调支架的安装</t>
-  </si>
-  <si>
-    <t xml:space="preserve">支架安装和紧固</t>
-  </si>
-  <si>
-    <t xml:space="preserve">型钢结构的支架，其紧固度</t>
+    <t>支架到场后检查</t>
+  </si>
+  <si>
+    <t>外观及防腐涂镀层</t>
+  </si>
+  <si>
+    <t>主控</t>
+  </si>
+  <si>
+    <t>完好无损</t>
+  </si>
+  <si>
+    <t>合格</t>
+  </si>
+  <si>
+    <t>型号、规格及材质</t>
+  </si>
+  <si>
+    <t>符合设计图纸要求，附件、备件应齐全</t>
+  </si>
+  <si>
+    <t>存放在滩涂、盐碱等腐蚀性强的场所的支架</t>
+  </si>
+  <si>
+    <t>做好防腐蚀工作</t>
+  </si>
+  <si>
+    <t>基础及预埋件（预埋螺栓）的水平偏差和定位轴线偏差</t>
+  </si>
+  <si>
+    <t>“中间交接验收签证书”的相关要求</t>
+  </si>
+  <si>
+    <t>固定式支架及手动可调支架的安装</t>
+  </si>
+  <si>
+    <t>支架安装和紧固</t>
+  </si>
+  <si>
+    <t>型钢结构的支架，其紧固度</t>
   </si>
   <si>
     <r>
@@ -310,60 +308,58 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">符合设计图纸要求及</t>
+      <t>符合设计图纸要求及</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">GB 50205</t>
+      <t>GB 50205</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">的相关规定</t>
+      <t>的相关规定</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">支架安装过程中</t>
-  </si>
-  <si>
-    <t xml:space="preserve">不应强行敲打，不应气割扩孔。对热镀锌材质的支架，现场不宜打孔</t>
-  </si>
-  <si>
-    <t xml:space="preserve">支架防腐层</t>
-  </si>
-  <si>
-    <t xml:space="preserve">不应破坏</t>
-  </si>
-  <si>
-    <t xml:space="preserve">手动可调式支架调整动作</t>
-  </si>
-  <si>
-    <t xml:space="preserve">灵活</t>
-  </si>
-  <si>
-    <t xml:space="preserve">高度角调节范围</t>
-  </si>
-  <si>
-    <t xml:space="preserve">满足设计要求</t>
-  </si>
-  <si>
-    <t xml:space="preserve">支架倾斜角度偏差度</t>
-  </si>
-  <si>
-    <t xml:space="preserve">一般</t>
+    <t>支架安装过程中</t>
+  </si>
+  <si>
+    <t>不应强行敲打，不应气割扩孔。对热镀锌材质的支架，现场不宜打孔</t>
+  </si>
+  <si>
+    <t>支架防腐层</t>
+  </si>
+  <si>
+    <t>不应破坏</t>
+  </si>
+  <si>
+    <t>手动可调式支架调整动作</t>
+  </si>
+  <si>
+    <t>灵活</t>
+  </si>
+  <si>
+    <t>高度角调节范围</t>
+  </si>
+  <si>
+    <t>满足设计要求</t>
+  </si>
+  <si>
+    <t>支架倾斜角度偏差度</t>
+  </si>
+  <si>
+    <t>一般</t>
   </si>
   <si>
     <r>
@@ -371,50 +367,49 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">不应大于</t>
+      <t>不应大于</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">±1°</t>
+      <t>±1°</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">0,0,1,0,0,0,1,0,0,1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">固定及手动可调支架安装的允许偏差</t>
-  </si>
-  <si>
-    <t xml:space="preserve">中心线偏差</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≤2mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,2,1,2,1,0,1,0,0,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">梁标高偏差（同组）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≤3mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,2,1,2,2,1,1,2,0,1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">立柱面偏差（同组）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,2,1,1,1,2,3,1,1,3</t>
+    <t>0,0,1,0,0,0,1,0,0,1</t>
+  </si>
+  <si>
+    <t>固定及手动可调支架安装的允许偏差</t>
+  </si>
+  <si>
+    <t>中心线偏差</t>
+  </si>
+  <si>
+    <t>≤2mm</t>
+  </si>
+  <si>
+    <t>1,2,1,2,1,0,1,0,0,2</t>
+  </si>
+  <si>
+    <t>梁标高偏差（同组）</t>
+  </si>
+  <si>
+    <t>≤3mm</t>
+  </si>
+  <si>
+    <t>0,2,1,2,2,1,1,2,0,1</t>
+  </si>
+  <si>
+    <t>立柱面偏差（同组）</t>
+  </si>
+  <si>
+    <t>0,2,1,1,1,2,3,1,1,3</t>
   </si>
   <si>
     <r>
@@ -422,17 +417,16 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">表</t>
+      <t>表</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
       <t xml:space="preserve">5.2 </t>
     </r>
@@ -441,53 +435,52 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">支架安装分项工程质量验收表</t>
+      <t>支架安装分项工程质量验收表</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">1#</t>
+      <t>1#</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">跟踪式支架的安装</t>
-  </si>
-  <si>
-    <t xml:space="preserve">跟踪式支架及基础之间</t>
-  </si>
-  <si>
-    <t xml:space="preserve">固定牢固、可靠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">跟踪式支架安装的允许偏差</t>
-  </si>
-  <si>
-    <t xml:space="preserve">符合设计文件的规定</t>
-  </si>
-  <si>
-    <t xml:space="preserve">跟踪式支架电机的安装</t>
-  </si>
-  <si>
-    <t xml:space="preserve">牢固、可靠。传动部分应动作灵活</t>
-  </si>
-  <si>
-    <t xml:space="preserve">聚光式跟踪系统的聚光部件安装完成后</t>
-  </si>
-  <si>
-    <t xml:space="preserve">采取相应防护措施</t>
-  </si>
-  <si>
-    <t xml:space="preserve">支架的现场焊接工艺</t>
-  </si>
-  <si>
-    <t xml:space="preserve">支架的组装、焊接与防腐处理</t>
+    <t>跟踪式支架的安装</t>
+  </si>
+  <si>
+    <t>跟踪式支架及基础之间</t>
+  </si>
+  <si>
+    <t>固定牢固、可靠</t>
+  </si>
+  <si>
+    <t>跟踪式支架安装的允许偏差</t>
+  </si>
+  <si>
+    <t>符合设计文件的规定</t>
+  </si>
+  <si>
+    <t>跟踪式支架电机的安装</t>
+  </si>
+  <si>
+    <t>牢固、可靠。传动部分应动作灵活</t>
+  </si>
+  <si>
+    <t>聚光式跟踪系统的聚光部件安装完成后</t>
+  </si>
+  <si>
+    <t>采取相应防护措施</t>
+  </si>
+  <si>
+    <t>支架的现场焊接工艺</t>
+  </si>
+  <si>
+    <t>支架的组装、焊接与防腐处理</t>
   </si>
   <si>
     <r>
@@ -495,123 +488,249 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">GB 50018</t>
+      <t>GB 50018</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">及</t>
+      <t>及</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
+        <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">GB 50017</t>
+      <t>GB 50017</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
-        <family val="0"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">的相关规定</t>
+      <t>的相关规定</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">焊接工作完毕后</t>
-  </si>
-  <si>
-    <t xml:space="preserve">对焊缝进行检查</t>
-  </si>
-  <si>
-    <t xml:space="preserve">支架安装完成后，其焊接表面</t>
-  </si>
-  <si>
-    <t xml:space="preserve">按照设计要求进行防腐处理</t>
+    <t>焊接工作完毕后</t>
+  </si>
+  <si>
+    <t>对焊缝进行检查</t>
+  </si>
+  <si>
+    <t>支架安装完成后，其焊接表面</t>
+  </si>
+  <si>
+    <t>按照设计要求进行防腐处理</t>
   </si>
   <si>
     <t xml:space="preserve"> 验收结论：</t>
   </si>
   <si>
-    <t xml:space="preserve">验收单位签字</t>
-  </si>
-  <si>
-    <t xml:space="preserve">年  月  日</t>
-  </si>
-  <si>
-    <t xml:space="preserve">监理单位</t>
+    <t>验收单位签字</t>
+  </si>
+  <si>
+    <t>年  月  日</t>
+  </si>
+  <si>
+    <t>监理单位</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="24">
     <font>
       <sz val="10"/>
       <name val="宋体"/>
-      <family val="0"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="宋体"/>
-      <family val="0"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="17"/>
       <color rgb="FF000000"/>
       <name val="黑体"/>
-      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="17"/>
-      <color rgb="FF000000"/>
-      <name val="黑体"/>
-      <family val="3"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="宋体"/>
-      <family val="0"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="DejaVu Sans"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="DejaVu Sans"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="DejaVu Sans"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="DejaVu Sans"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="DejaVu Sans"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="DejaVu Sans"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -624,289 +743,997 @@
         <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
-    <border diagonalUp="false" diagonalDown="false">
+  <borders count="24">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="thin"/>
-      <top style="medium"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="medium"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top style="medium"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="medium"/>
-      <top style="thin"/>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="medium"/>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
-      <right style="medium"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellXfs count="27">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color theme="4"/>
+        </left>
+        <right style="thin">
+          <color theme="4"/>
+        </right>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <horizontal style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    </tableStyle>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
@@ -948,17 +1775,17 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1008,30 +1835,31 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="true"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AJ25"/>
-  <sheetFormatPr defaultColWidth="9.2109375" defaultRowHeight="13" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.20952380952381" defaultRowHeight="12"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="0.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="2.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="0" width="3.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="2.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="14" style="0" width="3.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="22" style="0" width="2.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="3.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="2.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="2.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="0.65"/>
+    <col min="1" max="1" width="0.647619047619048" customWidth="1"/>
+    <col min="2" max="5" width="2.87619047619048" customWidth="1"/>
+    <col min="6" max="11" width="3.31428571428571" customWidth="1"/>
+    <col min="12" max="13" width="2.87619047619048" customWidth="1"/>
+    <col min="14" max="21" width="3.31428571428571" customWidth="1"/>
+    <col min="22" max="31" width="2.87619047619048" customWidth="1"/>
+    <col min="32" max="32" width="3.31428571428571" customWidth="1"/>
+    <col min="33" max="33" width="2.54285714285714" customWidth="1"/>
+    <col min="34" max="34" width="2.64761904761905" customWidth="1"/>
+    <col min="35" max="35" width="0.647619047619048" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" ht="3.75" customHeight="1" spans="1:36">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1068,7 +1896,7 @@
       <c r="AH1" s="1"/>
       <c r="AI1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" ht="22.5" customHeight="1" spans="1:36">
       <c r="A2" s="1"/>
       <c r="B2" s="3" t="s">
         <v>0</v>
@@ -1107,7 +1935,7 @@
       <c r="AH2" s="3"/>
       <c r="AI2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" ht="22.5" customHeight="1" spans="1:36">
       <c r="A3" s="1"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1144,90 +1972,90 @@
       <c r="AH3" s="3"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="24.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" ht="24.6" customHeight="1" spans="1:36">
       <c r="A4" s="1"/>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
-      <c r="AA4" s="5"/>
-      <c r="AB4" s="4" t="s">
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
+      <c r="X4" s="21"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="21"/>
+      <c r="AA4" s="21"/>
+      <c r="AB4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="AC4" s="4"/>
-      <c r="AD4" s="4"/>
-      <c r="AE4" s="4"/>
-      <c r="AF4" s="4"/>
-      <c r="AG4" s="4"/>
-      <c r="AH4" s="4"/>
+      <c r="AC4" s="6"/>
+      <c r="AD4" s="6"/>
+      <c r="AE4" s="6"/>
+      <c r="AF4" s="6"/>
+      <c r="AG4" s="6"/>
+      <c r="AH4" s="6"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" ht="33.75" customHeight="1" spans="1:36">
       <c r="A5" s="1"/>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="7" t="s">
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7" t="s">
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
-      <c r="R5" s="7"/>
-      <c r="S5" s="7"/>
-      <c r="T5" s="7" t="s">
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
+      <c r="T5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="U5" s="7"/>
-      <c r="V5" s="7"/>
-      <c r="W5" s="7"/>
-      <c r="X5" s="7"/>
-      <c r="Y5" s="7"/>
-      <c r="Z5" s="7" t="s">
+      <c r="U5" s="8"/>
+      <c r="V5" s="8"/>
+      <c r="W5" s="8"/>
+      <c r="X5" s="8"/>
+      <c r="Y5" s="8"/>
+      <c r="Z5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="AA5" s="7"/>
-      <c r="AB5" s="7"/>
-      <c r="AC5" s="7"/>
-      <c r="AD5" s="7"/>
+      <c r="AA5" s="8"/>
+      <c r="AB5" s="8"/>
+      <c r="AC5" s="8"/>
+      <c r="AD5" s="8"/>
       <c r="AE5" s="8" t="s">
         <v>9</v>
       </c>
@@ -1237,7 +2065,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="9"/>
     </row>
-    <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" ht="33.75" customHeight="1" spans="1:36">
       <c r="A6" s="1"/>
       <c r="B6" s="10" t="s">
         <v>10</v>
@@ -1287,7 +2115,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="9"/>
     </row>
-    <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" ht="33.75" customHeight="1" spans="1:36">
       <c r="A7" s="1"/>
       <c r="B7" s="10" t="s">
         <v>16</v>
@@ -1337,7 +2165,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="9"/>
     </row>
-    <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" ht="33.75" customHeight="1" spans="1:36">
       <c r="A8" s="1"/>
       <c r="B8" s="10" t="s">
         <v>18</v>
@@ -1385,7 +2213,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="9"/>
     </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" ht="30" customHeight="1" spans="1:36">
       <c r="A9" s="1"/>
       <c r="B9" s="10" t="s">
         <v>23</v>
@@ -1434,7 +2262,7 @@
       <c r="AH9" s="12"/>
       <c r="AI9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" ht="48.75" customHeight="1" spans="1:36">
       <c r="A10" s="1"/>
       <c r="B10" s="10" t="s">
         <v>29</v>
@@ -1474,14 +2302,14 @@
       <c r="AC10" s="11"/>
       <c r="AD10" s="11"/>
       <c r="AE10" s="11"/>
-      <c r="AF10" s="14" t="s">
+      <c r="AF10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG10" s="14"/>
-      <c r="AH10" s="14"/>
+      <c r="AG10" s="12"/>
+      <c r="AH10" s="12"/>
       <c r="AI10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" ht="48.75" customHeight="1" spans="1:36">
       <c r="A11" s="1"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -1530,7 +2358,7 @@
       <c r="AH11" s="12"/>
       <c r="AI11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" ht="48.75" customHeight="1" spans="1:36">
       <c r="A12" s="1"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -1577,7 +2405,7 @@
       <c r="AH12" s="12"/>
       <c r="AI12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" ht="48.75" customHeight="1" spans="1:36">
       <c r="A13" s="1"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1615,14 +2443,14 @@
       <c r="AC13" s="11"/>
       <c r="AD13" s="11"/>
       <c r="AE13" s="11"/>
-      <c r="AF13" s="14" t="s">
+      <c r="AF13" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG13" s="14"/>
-      <c r="AH13" s="14"/>
+      <c r="AG13" s="12"/>
+      <c r="AH13" s="12"/>
       <c r="AI13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" ht="48.75" customHeight="1" spans="1:36">
       <c r="A14" s="1"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -1638,16 +2466,16 @@
       <c r="K14" s="13"/>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
-      <c r="N14" s="15" t="s">
+      <c r="N14" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15"/>
-      <c r="Q14" s="15"/>
-      <c r="R14" s="15"/>
-      <c r="S14" s="15"/>
-      <c r="T14" s="15"/>
-      <c r="U14" s="15"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="22"/>
+      <c r="Q14" s="22"/>
+      <c r="R14" s="22"/>
+      <c r="S14" s="22"/>
+      <c r="T14" s="22"/>
+      <c r="U14" s="22"/>
       <c r="V14" s="11" t="s">
         <v>32</v>
       </c>
@@ -1660,21 +2488,21 @@
       <c r="AC14" s="11"/>
       <c r="AD14" s="11"/>
       <c r="AE14" s="11"/>
-      <c r="AF14" s="14" t="s">
+      <c r="AF14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG14" s="14"/>
-      <c r="AH14" s="14"/>
+      <c r="AG14" s="12"/>
+      <c r="AH14" s="12"/>
       <c r="AI14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" ht="48.75" customHeight="1" spans="1:36">
       <c r="A15" s="1"/>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
       <c r="F15" s="11" t="s">
         <v>45</v>
       </c>
@@ -1718,12 +2546,12 @@
       <c r="AH15" s="12"/>
       <c r="AI15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" ht="48.75" customHeight="1" spans="1:36">
       <c r="A16" s="1"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
       <c r="H16" s="13" t="s">
@@ -1765,12 +2593,12 @@
       <c r="AH16" s="12"/>
       <c r="AI16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" ht="48.75" customHeight="1" spans="1:35">
       <c r="A17" s="1"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
       <c r="F17" s="11"/>
       <c r="G17" s="11"/>
       <c r="H17" s="13" t="s">
@@ -1783,16 +2611,16 @@
         <v>35</v>
       </c>
       <c r="M17" s="11"/>
-      <c r="N17" s="15" t="s">
+      <c r="N17" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="O17" s="15"/>
-      <c r="P17" s="15"/>
-      <c r="Q17" s="15"/>
-      <c r="R17" s="15"/>
-      <c r="S17" s="15"/>
-      <c r="T17" s="15"/>
-      <c r="U17" s="15"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="22"/>
+      <c r="Q17" s="22"/>
+      <c r="R17" s="22"/>
+      <c r="S17" s="22"/>
+      <c r="T17" s="22"/>
+      <c r="U17" s="22"/>
       <c r="V17" s="11" t="s">
         <v>32</v>
       </c>
@@ -1812,12 +2640,12 @@
       <c r="AH17" s="12"/>
       <c r="AI17" s="2"/>
     </row>
-    <row r="18" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" ht="48.75" customHeight="1" spans="1:35">
       <c r="A18" s="1"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
       <c r="H18" s="13" t="s">
@@ -1850,19 +2678,19 @@
       <c r="AC18" s="11"/>
       <c r="AD18" s="11"/>
       <c r="AE18" s="11"/>
-      <c r="AF18" s="14" t="s">
+      <c r="AF18" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG18" s="14"/>
-      <c r="AH18" s="14"/>
+      <c r="AG18" s="12"/>
+      <c r="AH18" s="12"/>
       <c r="AI18" s="2"/>
     </row>
-    <row r="19" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" ht="48.75" customHeight="1" spans="1:35">
       <c r="A19" s="1"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
       <c r="H19" s="13" t="s">
@@ -1895,19 +2723,19 @@
       <c r="AC19" s="11"/>
       <c r="AD19" s="11"/>
       <c r="AE19" s="11"/>
-      <c r="AF19" s="14" t="s">
+      <c r="AF19" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG19" s="14"/>
-      <c r="AH19" s="14"/>
+      <c r="AG19" s="12"/>
+      <c r="AH19" s="12"/>
       <c r="AI19" s="2"/>
     </row>
-    <row r="20" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" ht="48.75" customHeight="1" spans="1:35">
       <c r="A20" s="1"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
       <c r="F20" s="13" t="s">
         <v>56</v>
       </c>
@@ -1930,18 +2758,18 @@
       <c r="S20" s="11"/>
       <c r="T20" s="11"/>
       <c r="U20" s="11"/>
-      <c r="V20" s="17" t="s">
+      <c r="V20" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="W20" s="17"/>
-      <c r="X20" s="17"/>
-      <c r="Y20" s="17"/>
-      <c r="Z20" s="17"/>
-      <c r="AA20" s="17"/>
-      <c r="AB20" s="17"/>
-      <c r="AC20" s="17"/>
-      <c r="AD20" s="17"/>
-      <c r="AE20" s="17"/>
+      <c r="W20" s="11"/>
+      <c r="X20" s="11"/>
+      <c r="Y20" s="11"/>
+      <c r="Z20" s="11"/>
+      <c r="AA20" s="11"/>
+      <c r="AB20" s="11"/>
+      <c r="AC20" s="11"/>
+      <c r="AD20" s="11"/>
+      <c r="AE20" s="11"/>
       <c r="AF20" s="12" t="s">
         <v>37</v>
       </c>
@@ -1949,16 +2777,16 @@
       <c r="AH20" s="12"/>
       <c r="AI20" s="2"/>
     </row>
-    <row r="21" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" ht="48.75" customHeight="1" spans="1:35">
       <c r="A21" s="1"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="18" t="s">
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="G21" s="18"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="13" t="s">
         <v>61</v>
       </c>
@@ -1969,28 +2797,28 @@
         <v>57</v>
       </c>
       <c r="M21" s="11"/>
-      <c r="N21" s="17" t="s">
+      <c r="N21" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="O21" s="17"/>
-      <c r="P21" s="17"/>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="17"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="17"/>
-      <c r="U21" s="17"/>
-      <c r="V21" s="17" t="s">
+      <c r="O21" s="11"/>
+      <c r="P21" s="11"/>
+      <c r="Q21" s="11"/>
+      <c r="R21" s="11"/>
+      <c r="S21" s="11"/>
+      <c r="T21" s="11"/>
+      <c r="U21" s="11"/>
+      <c r="V21" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="W21" s="17"/>
-      <c r="X21" s="17"/>
-      <c r="Y21" s="17"/>
-      <c r="Z21" s="17"/>
-      <c r="AA21" s="17"/>
-      <c r="AB21" s="17"/>
-      <c r="AC21" s="17"/>
-      <c r="AD21" s="17"/>
-      <c r="AE21" s="17"/>
+      <c r="W21" s="11"/>
+      <c r="X21" s="11"/>
+      <c r="Y21" s="11"/>
+      <c r="Z21" s="11"/>
+      <c r="AA21" s="11"/>
+      <c r="AB21" s="11"/>
+      <c r="AC21" s="11"/>
+      <c r="AD21" s="11"/>
+      <c r="AE21" s="11"/>
       <c r="AF21" s="12" t="s">
         <v>37</v>
       </c>
@@ -1998,14 +2826,14 @@
       <c r="AH21" s="12"/>
       <c r="AI21" s="2"/>
     </row>
-    <row r="22" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" ht="53.25" customHeight="1" spans="1:35">
       <c r="A22" s="1"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
       <c r="H22" s="13" t="s">
         <v>64</v>
       </c>
@@ -2016,28 +2844,28 @@
         <v>57</v>
       </c>
       <c r="M22" s="11"/>
-      <c r="N22" s="17" t="s">
+      <c r="N22" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="O22" s="17"/>
-      <c r="P22" s="17"/>
-      <c r="Q22" s="17"/>
-      <c r="R22" s="17"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="17"/>
-      <c r="U22" s="17"/>
-      <c r="V22" s="17" t="s">
+      <c r="O22" s="11"/>
+      <c r="P22" s="11"/>
+      <c r="Q22" s="11"/>
+      <c r="R22" s="11"/>
+      <c r="S22" s="11"/>
+      <c r="T22" s="11"/>
+      <c r="U22" s="11"/>
+      <c r="V22" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="W22" s="17"/>
-      <c r="X22" s="17"/>
-      <c r="Y22" s="17"/>
-      <c r="Z22" s="17"/>
-      <c r="AA22" s="17"/>
-      <c r="AB22" s="17"/>
-      <c r="AC22" s="17"/>
-      <c r="AD22" s="17"/>
-      <c r="AE22" s="17"/>
+      <c r="W22" s="11"/>
+      <c r="X22" s="11"/>
+      <c r="Y22" s="11"/>
+      <c r="Z22" s="11"/>
+      <c r="AA22" s="11"/>
+      <c r="AB22" s="11"/>
+      <c r="AC22" s="11"/>
+      <c r="AD22" s="11"/>
+      <c r="AE22" s="11"/>
       <c r="AF22" s="12" t="s">
         <v>37</v>
       </c>
@@ -2045,91 +2873,91 @@
       <c r="AH22" s="12"/>
       <c r="AI22" s="2"/>
     </row>
-    <row r="23" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" ht="46.5" customHeight="1" spans="1:35">
       <c r="A23" s="1"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="19" t="s">
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="18" t="s">
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="M23" s="18"/>
-      <c r="N23" s="20" t="s">
+      <c r="M23" s="24"/>
+      <c r="N23" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="O23" s="20"/>
-      <c r="P23" s="20"/>
-      <c r="Q23" s="20"/>
-      <c r="R23" s="20"/>
-      <c r="S23" s="20"/>
-      <c r="T23" s="20"/>
-      <c r="U23" s="20"/>
-      <c r="V23" s="20" t="s">
+      <c r="O23" s="24"/>
+      <c r="P23" s="24"/>
+      <c r="Q23" s="24"/>
+      <c r="R23" s="24"/>
+      <c r="S23" s="24"/>
+      <c r="T23" s="24"/>
+      <c r="U23" s="24"/>
+      <c r="V23" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="W23" s="20"/>
-      <c r="X23" s="20"/>
-      <c r="Y23" s="20"/>
-      <c r="Z23" s="20"/>
-      <c r="AA23" s="20"/>
-      <c r="AB23" s="20"/>
-      <c r="AC23" s="20"/>
-      <c r="AD23" s="20"/>
-      <c r="AE23" s="20"/>
-      <c r="AF23" s="21" t="s">
+      <c r="W23" s="24"/>
+      <c r="X23" s="24"/>
+      <c r="Y23" s="24"/>
+      <c r="Z23" s="24"/>
+      <c r="AA23" s="24"/>
+      <c r="AB23" s="24"/>
+      <c r="AC23" s="24"/>
+      <c r="AD23" s="24"/>
+      <c r="AE23" s="24"/>
+      <c r="AF23" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="AG23" s="21"/>
-      <c r="AH23" s="21"/>
+      <c r="AG23" s="26"/>
+      <c r="AH23" s="26"/>
       <c r="AI23" s="2"/>
     </row>
-    <row r="24" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" ht="3.75" customHeight="1" spans="1:35">
       <c r="A24" s="1"/>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
-      <c r="N24" s="22"/>
-      <c r="O24" s="22"/>
-      <c r="P24" s="22"/>
-      <c r="Q24" s="22"/>
-      <c r="R24" s="22"/>
-      <c r="S24" s="22"/>
-      <c r="T24" s="22"/>
-      <c r="U24" s="22"/>
-      <c r="V24" s="22"/>
-      <c r="W24" s="22"/>
-      <c r="X24" s="22"/>
-      <c r="Y24" s="22"/>
-      <c r="Z24" s="22"/>
-      <c r="AA24" s="22"/>
-      <c r="AB24" s="22"/>
-      <c r="AC24" s="22"/>
-      <c r="AD24" s="22"/>
-      <c r="AE24" s="22"/>
-      <c r="AF24" s="22"/>
-      <c r="AG24" s="22"/>
-      <c r="AH24" s="22"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="19"/>
+      <c r="O24" s="19"/>
+      <c r="P24" s="19"/>
+      <c r="Q24" s="19"/>
+      <c r="R24" s="19"/>
+      <c r="S24" s="19"/>
+      <c r="T24" s="19"/>
+      <c r="U24" s="19"/>
+      <c r="V24" s="19"/>
+      <c r="W24" s="19"/>
+      <c r="X24" s="19"/>
+      <c r="Y24" s="19"/>
+      <c r="Z24" s="19"/>
+      <c r="AA24" s="19"/>
+      <c r="AB24" s="19"/>
+      <c r="AC24" s="19"/>
+      <c r="AD24" s="19"/>
+      <c r="AE24" s="19"/>
+      <c r="AF24" s="19"/>
+      <c r="AG24" s="19"/>
+      <c r="AH24" s="19"/>
       <c r="AI24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="409.5" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" ht="409.5" hidden="1" customHeight="1" spans="1:35">
       <c r="A25" s="1" t="s">
         <v>69</v>
       </c>
@@ -2166,14 +2994,11 @@
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
       <c r="AH25" s="1"/>
-      <c r="AI25" s="23"/>
+      <c r="AI25" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="114">
-    <mergeCell ref="A1:A24"/>
     <mergeCell ref="B1:AH1"/>
-    <mergeCell ref="AI1:AI23"/>
-    <mergeCell ref="B2:AH3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="F4:U4"/>
     <mergeCell ref="AB4:AH4"/>
@@ -2207,13 +3032,11 @@
     <mergeCell ref="N9:U9"/>
     <mergeCell ref="V9:AE9"/>
     <mergeCell ref="AF9:AH9"/>
-    <mergeCell ref="B10:E14"/>
     <mergeCell ref="F10:K10"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="N10:U10"/>
     <mergeCell ref="V10:AE10"/>
     <mergeCell ref="AF10:AH10"/>
-    <mergeCell ref="F11:G14"/>
     <mergeCell ref="H11:K11"/>
     <mergeCell ref="L11:M11"/>
     <mergeCell ref="N11:U11"/>
@@ -2234,8 +3057,6 @@
     <mergeCell ref="N14:U14"/>
     <mergeCell ref="V14:AE14"/>
     <mergeCell ref="AF14:AH14"/>
-    <mergeCell ref="B15:E23"/>
-    <mergeCell ref="F15:G19"/>
     <mergeCell ref="H15:K15"/>
     <mergeCell ref="L15:M15"/>
     <mergeCell ref="N15:U15"/>
@@ -2266,7 +3087,6 @@
     <mergeCell ref="N20:U20"/>
     <mergeCell ref="V20:AE20"/>
     <mergeCell ref="AF20:AH20"/>
-    <mergeCell ref="F21:G23"/>
     <mergeCell ref="H21:K21"/>
     <mergeCell ref="L21:M21"/>
     <mergeCell ref="N21:U21"/>
@@ -2284,38 +3104,43 @@
     <mergeCell ref="AF23:AH23"/>
     <mergeCell ref="B24:AH24"/>
     <mergeCell ref="A25:AH25"/>
+    <mergeCell ref="A1:A24"/>
+    <mergeCell ref="AI1:AI23"/>
+    <mergeCell ref="B2:AH3"/>
+    <mergeCell ref="B10:E14"/>
+    <mergeCell ref="F11:G14"/>
+    <mergeCell ref="B15:E23"/>
+    <mergeCell ref="F15:G19"/>
+    <mergeCell ref="F21:G23"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0" top="0.590277777777778" bottom="0" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0" right="0" top="0.590277777777778" bottom="0" header="0.511805555555556" footer="0.511805555555556"/>
+  <pageSetup paperSize="9" scale="82" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="true"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AJ28"/>
-  <sheetFormatPr defaultColWidth="9.2109375" defaultRowHeight="13" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.20952380952381" defaultRowHeight="12"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="0.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="2.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="0" width="3.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="2.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="14" style="0" width="3.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="22" style="0" width="2.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="3.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="2.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="2.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="0.65"/>
+    <col min="1" max="1" width="0.647619047619048" customWidth="1"/>
+    <col min="2" max="5" width="2.87619047619048" customWidth="1"/>
+    <col min="6" max="11" width="3.31428571428571" customWidth="1"/>
+    <col min="12" max="13" width="2.87619047619048" customWidth="1"/>
+    <col min="14" max="21" width="3.31428571428571" customWidth="1"/>
+    <col min="22" max="31" width="2.87619047619048" customWidth="1"/>
+    <col min="32" max="32" width="3.31428571428571" customWidth="1"/>
+    <col min="33" max="33" width="2.54285714285714" customWidth="1"/>
+    <col min="34" max="34" width="2.64761904761905" customWidth="1"/>
+    <col min="35" max="35" width="0.647619047619048" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" ht="3.75" customHeight="1" spans="1:36">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2352,7 +3177,7 @@
       <c r="AH1" s="1"/>
       <c r="AI1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" ht="22.5" customHeight="1" spans="1:36">
       <c r="A2" s="1"/>
       <c r="B2" s="3" t="s">
         <v>0</v>
@@ -2391,7 +3216,7 @@
       <c r="AH2" s="3"/>
       <c r="AI2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" ht="22.5" customHeight="1" spans="1:36">
       <c r="A3" s="1"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -2428,7 +3253,7 @@
       <c r="AH3" s="3"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" ht="26.25" customHeight="1" spans="1:36">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
@@ -2436,119 +3261,119 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
-      <c r="N4" s="24"/>
-      <c r="O4" s="24"/>
-      <c r="P4" s="24"/>
-      <c r="Q4" s="24"/>
-      <c r="R4" s="24"/>
-      <c r="S4" s="24"/>
-      <c r="T4" s="24"/>
-      <c r="U4" s="24"/>
-      <c r="V4" s="24"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
-      <c r="AA4" s="25" t="s">
+      <c r="AA4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="AB4" s="25"/>
-      <c r="AC4" s="25"/>
-      <c r="AD4" s="25"/>
-      <c r="AE4" s="25"/>
-      <c r="AF4" s="25"/>
-      <c r="AG4" s="25"/>
-      <c r="AH4" s="25"/>
+      <c r="AB4" s="5"/>
+      <c r="AC4" s="5"/>
+      <c r="AD4" s="5"/>
+      <c r="AE4" s="5"/>
+      <c r="AF4" s="5"/>
+      <c r="AG4" s="5"/>
+      <c r="AH4" s="5"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" ht="3.75" customHeight="1" spans="1:36">
       <c r="A5" s="1"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
-      <c r="Z5" s="4"/>
-      <c r="AA5" s="4"/>
-      <c r="AB5" s="4"/>
-      <c r="AC5" s="4"/>
-      <c r="AD5" s="4"/>
-      <c r="AE5" s="4"/>
-      <c r="AF5" s="4"/>
-      <c r="AG5" s="4"/>
-      <c r="AH5" s="4"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+      <c r="X5" s="6"/>
+      <c r="Y5" s="6"/>
+      <c r="Z5" s="6"/>
+      <c r="AA5" s="6"/>
+      <c r="AB5" s="6"/>
+      <c r="AC5" s="6"/>
+      <c r="AD5" s="6"/>
+      <c r="AE5" s="6"/>
+      <c r="AF5" s="6"/>
+      <c r="AG5" s="6"/>
+      <c r="AH5" s="6"/>
       <c r="AI5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" ht="33.75" customHeight="1" spans="1:36">
       <c r="A6" s="1"/>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="7" t="s">
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7" t="s">
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7"/>
-      <c r="R6" s="7"/>
-      <c r="S6" s="7"/>
-      <c r="T6" s="7" t="s">
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="U6" s="7"/>
-      <c r="V6" s="7"/>
-      <c r="W6" s="7"/>
-      <c r="X6" s="7"/>
-      <c r="Y6" s="7"/>
-      <c r="Z6" s="7" t="s">
+      <c r="U6" s="8"/>
+      <c r="V6" s="8"/>
+      <c r="W6" s="8"/>
+      <c r="X6" s="8"/>
+      <c r="Y6" s="8"/>
+      <c r="Z6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="AA6" s="7"/>
-      <c r="AB6" s="7"/>
-      <c r="AC6" s="7"/>
-      <c r="AD6" s="7"/>
+      <c r="AA6" s="8"/>
+      <c r="AB6" s="8"/>
+      <c r="AC6" s="8"/>
+      <c r="AD6" s="8"/>
       <c r="AE6" s="8" t="s">
         <v>9</v>
       </c>
@@ -2558,7 +3383,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="9"/>
     </row>
-    <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" ht="33.75" customHeight="1" spans="1:36">
       <c r="A7" s="1"/>
       <c r="B7" s="10" t="s">
         <v>10</v>
@@ -2608,7 +3433,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="9"/>
     </row>
-    <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" ht="33.75" customHeight="1" spans="1:36">
       <c r="A8" s="1"/>
       <c r="B8" s="10" t="s">
         <v>16</v>
@@ -2658,7 +3483,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="9"/>
     </row>
-    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" ht="33.75" customHeight="1" spans="1:36">
       <c r="A9" s="1"/>
       <c r="B9" s="10" t="s">
         <v>18</v>
@@ -2706,7 +3531,7 @@
       <c r="AI9" s="2"/>
       <c r="AJ9" s="9"/>
     </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" ht="30" customHeight="1" spans="1:36">
       <c r="A10" s="1"/>
       <c r="B10" s="10" t="s">
         <v>23</v>
@@ -2755,7 +3580,7 @@
       <c r="AH10" s="12"/>
       <c r="AI10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" ht="56.25" customHeight="1" spans="1:36">
       <c r="A11" s="1"/>
       <c r="B11" s="10" t="s">
         <v>70</v>
@@ -2795,14 +3620,14 @@
       <c r="AC11" s="11"/>
       <c r="AD11" s="11"/>
       <c r="AE11" s="11"/>
-      <c r="AF11" s="14" t="s">
+      <c r="AF11" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG11" s="14"/>
-      <c r="AH11" s="14"/>
+      <c r="AG11" s="12"/>
+      <c r="AH11" s="12"/>
       <c r="AI11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" ht="56.25" customHeight="1" spans="1:36">
       <c r="A12" s="1"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -2840,14 +3665,14 @@
       <c r="AC12" s="11"/>
       <c r="AD12" s="11"/>
       <c r="AE12" s="11"/>
-      <c r="AF12" s="14" t="s">
+      <c r="AF12" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG12" s="14"/>
-      <c r="AH12" s="14"/>
+      <c r="AG12" s="12"/>
+      <c r="AH12" s="12"/>
       <c r="AI12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" ht="55.5" customHeight="1" spans="1:36">
       <c r="A13" s="1"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -2885,14 +3710,14 @@
       <c r="AC13" s="11"/>
       <c r="AD13" s="11"/>
       <c r="AE13" s="11"/>
-      <c r="AF13" s="14" t="s">
+      <c r="AF13" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG13" s="14"/>
-      <c r="AH13" s="14"/>
+      <c r="AG13" s="12"/>
+      <c r="AH13" s="12"/>
       <c r="AI13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" ht="55.5" customHeight="1" spans="1:36">
       <c r="A14" s="1"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -2930,14 +3755,14 @@
       <c r="AC14" s="11"/>
       <c r="AD14" s="11"/>
       <c r="AE14" s="11"/>
-      <c r="AF14" s="14" t="s">
+      <c r="AF14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG14" s="14"/>
-      <c r="AH14" s="14"/>
+      <c r="AG14" s="12"/>
+      <c r="AH14" s="12"/>
       <c r="AI14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" ht="55.5" customHeight="1" spans="1:36">
       <c r="A15" s="1"/>
       <c r="B15" s="10" t="s">
         <v>79</v>
@@ -2955,16 +3780,16 @@
       <c r="K15" s="13"/>
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
-      <c r="N15" s="26" t="s">
+      <c r="N15" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="O15" s="26"/>
-      <c r="P15" s="26"/>
-      <c r="Q15" s="26"/>
-      <c r="R15" s="26"/>
-      <c r="S15" s="26"/>
-      <c r="T15" s="26"/>
-      <c r="U15" s="26"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="13"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="13"/>
+      <c r="S15" s="13"/>
+      <c r="T15" s="13"/>
+      <c r="U15" s="13"/>
       <c r="V15" s="11" t="s">
         <v>32</v>
       </c>
@@ -2977,14 +3802,14 @@
       <c r="AC15" s="11"/>
       <c r="AD15" s="11"/>
       <c r="AE15" s="11"/>
-      <c r="AF15" s="14" t="s">
+      <c r="AF15" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG15" s="14"/>
-      <c r="AH15" s="14"/>
+      <c r="AG15" s="12"/>
+      <c r="AH15" s="12"/>
       <c r="AI15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" ht="55.5" customHeight="1" spans="1:36">
       <c r="A16" s="1"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -3022,14 +3847,14 @@
       <c r="AC16" s="11"/>
       <c r="AD16" s="11"/>
       <c r="AE16" s="11"/>
-      <c r="AF16" s="14" t="s">
+      <c r="AF16" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG16" s="14"/>
-      <c r="AH16" s="14"/>
+      <c r="AG16" s="12"/>
+      <c r="AH16" s="12"/>
       <c r="AI16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" ht="55.5" customHeight="1" spans="1:35">
       <c r="A17" s="1"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -3067,240 +3892,240 @@
       <c r="AC17" s="11"/>
       <c r="AD17" s="11"/>
       <c r="AE17" s="11"/>
-      <c r="AF17" s="14" t="s">
+      <c r="AF17" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="AG17" s="14"/>
-      <c r="AH17" s="14"/>
+      <c r="AG17" s="12"/>
+      <c r="AH17" s="12"/>
       <c r="AI17" s="2"/>
     </row>
-    <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" ht="26.25" customHeight="1" spans="1:35">
       <c r="A18" s="1"/>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="27"/>
-      <c r="M18" s="27"/>
-      <c r="N18" s="27"/>
-      <c r="O18" s="27"/>
-      <c r="P18" s="27"/>
-      <c r="Q18" s="27"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
-      <c r="V18" s="27"/>
-      <c r="W18" s="27"/>
-      <c r="X18" s="27"/>
-      <c r="Y18" s="27"/>
-      <c r="Z18" s="27"/>
-      <c r="AA18" s="27"/>
-      <c r="AB18" s="27"/>
-      <c r="AC18" s="27"/>
-      <c r="AD18" s="27"/>
-      <c r="AE18" s="27"/>
-      <c r="AF18" s="27"/>
-      <c r="AG18" s="27"/>
-      <c r="AH18" s="27"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="14"/>
+      <c r="T18" s="14"/>
+      <c r="U18" s="14"/>
+      <c r="V18" s="14"/>
+      <c r="W18" s="14"/>
+      <c r="X18" s="14"/>
+      <c r="Y18" s="14"/>
+      <c r="Z18" s="14"/>
+      <c r="AA18" s="14"/>
+      <c r="AB18" s="14"/>
+      <c r="AC18" s="14"/>
+      <c r="AD18" s="14"/>
+      <c r="AE18" s="14"/>
+      <c r="AF18" s="14"/>
+      <c r="AG18" s="14"/>
+      <c r="AH18" s="14"/>
       <c r="AI18" s="2"/>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" ht="30" customHeight="1" spans="1:35">
       <c r="A19" s="1"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
-      <c r="L19" s="28"/>
-      <c r="M19" s="28"/>
-      <c r="N19" s="28"/>
-      <c r="O19" s="28"/>
-      <c r="P19" s="28"/>
-      <c r="Q19" s="28"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
-      <c r="V19" s="28"/>
-      <c r="W19" s="28"/>
-      <c r="X19" s="28"/>
-      <c r="Y19" s="28"/>
-      <c r="Z19" s="28"/>
-      <c r="AA19" s="28"/>
-      <c r="AB19" s="28"/>
-      <c r="AC19" s="28"/>
-      <c r="AD19" s="28"/>
-      <c r="AE19" s="28"/>
-      <c r="AF19" s="28"/>
-      <c r="AG19" s="28"/>
-      <c r="AH19" s="28"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="15"/>
+      <c r="P19" s="15"/>
+      <c r="Q19" s="15"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="15"/>
+      <c r="T19" s="15"/>
+      <c r="U19" s="15"/>
+      <c r="V19" s="15"/>
+      <c r="W19" s="15"/>
+      <c r="X19" s="15"/>
+      <c r="Y19" s="15"/>
+      <c r="Z19" s="15"/>
+      <c r="AA19" s="15"/>
+      <c r="AB19" s="15"/>
+      <c r="AC19" s="15"/>
+      <c r="AD19" s="15"/>
+      <c r="AE19" s="15"/>
+      <c r="AF19" s="15"/>
+      <c r="AG19" s="15"/>
+      <c r="AH19" s="15"/>
       <c r="AI19" s="2"/>
     </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" ht="30" customHeight="1" spans="1:35">
       <c r="A20" s="1"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28"/>
-      <c r="P20" s="28"/>
-      <c r="Q20" s="28"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
-      <c r="T20" s="28"/>
-      <c r="U20" s="28"/>
-      <c r="V20" s="28"/>
-      <c r="W20" s="28"/>
-      <c r="X20" s="28"/>
-      <c r="Y20" s="28"/>
-      <c r="Z20" s="28"/>
-      <c r="AA20" s="28"/>
-      <c r="AB20" s="28"/>
-      <c r="AC20" s="28"/>
-      <c r="AD20" s="28"/>
-      <c r="AE20" s="28"/>
-      <c r="AF20" s="28"/>
-      <c r="AG20" s="28"/>
-      <c r="AH20" s="28"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15"/>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="15"/>
+      <c r="S20" s="15"/>
+      <c r="T20" s="15"/>
+      <c r="U20" s="15"/>
+      <c r="V20" s="15"/>
+      <c r="W20" s="15"/>
+      <c r="X20" s="15"/>
+      <c r="Y20" s="15"/>
+      <c r="Z20" s="15"/>
+      <c r="AA20" s="15"/>
+      <c r="AB20" s="15"/>
+      <c r="AC20" s="15"/>
+      <c r="AD20" s="15"/>
+      <c r="AE20" s="15"/>
+      <c r="AF20" s="15"/>
+      <c r="AG20" s="15"/>
+      <c r="AH20" s="15"/>
       <c r="AI20" s="2"/>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" ht="30" customHeight="1" spans="1:35">
       <c r="A21" s="1"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="28"/>
-      <c r="P21" s="28"/>
-      <c r="Q21" s="28"/>
-      <c r="R21" s="28"/>
-      <c r="S21" s="28"/>
-      <c r="T21" s="28"/>
-      <c r="U21" s="28"/>
-      <c r="V21" s="28"/>
-      <c r="W21" s="28"/>
-      <c r="X21" s="28"/>
-      <c r="Y21" s="28"/>
-      <c r="Z21" s="28"/>
-      <c r="AA21" s="28"/>
-      <c r="AB21" s="28"/>
-      <c r="AC21" s="28"/>
-      <c r="AD21" s="28"/>
-      <c r="AE21" s="28"/>
-      <c r="AF21" s="28"/>
-      <c r="AG21" s="28"/>
-      <c r="AH21" s="28"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="15"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
+      <c r="P21" s="15"/>
+      <c r="Q21" s="15"/>
+      <c r="R21" s="15"/>
+      <c r="S21" s="15"/>
+      <c r="T21" s="15"/>
+      <c r="U21" s="15"/>
+      <c r="V21" s="15"/>
+      <c r="W21" s="15"/>
+      <c r="X21" s="15"/>
+      <c r="Y21" s="15"/>
+      <c r="Z21" s="15"/>
+      <c r="AA21" s="15"/>
+      <c r="AB21" s="15"/>
+      <c r="AC21" s="15"/>
+      <c r="AD21" s="15"/>
+      <c r="AE21" s="15"/>
+      <c r="AF21" s="15"/>
+      <c r="AG21" s="15"/>
+      <c r="AH21" s="15"/>
       <c r="AI21" s="2"/>
     </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" ht="30" customHeight="1" spans="1:35">
       <c r="A22" s="1"/>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="28"/>
-      <c r="K22" s="28"/>
-      <c r="L22" s="28"/>
-      <c r="M22" s="28"/>
-      <c r="N22" s="28"/>
-      <c r="O22" s="28"/>
-      <c r="P22" s="28"/>
-      <c r="Q22" s="28"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-      <c r="U22" s="28"/>
-      <c r="V22" s="28"/>
-      <c r="W22" s="28"/>
-      <c r="X22" s="28"/>
-      <c r="Y22" s="28"/>
-      <c r="Z22" s="28"/>
-      <c r="AA22" s="28"/>
-      <c r="AB22" s="28"/>
-      <c r="AC22" s="28"/>
-      <c r="AD22" s="28"/>
-      <c r="AE22" s="28"/>
-      <c r="AF22" s="28"/>
-      <c r="AG22" s="28"/>
-      <c r="AH22" s="28"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+      <c r="O22" s="15"/>
+      <c r="P22" s="15"/>
+      <c r="Q22" s="15"/>
+      <c r="R22" s="15"/>
+      <c r="S22" s="15"/>
+      <c r="T22" s="15"/>
+      <c r="U22" s="15"/>
+      <c r="V22" s="15"/>
+      <c r="W22" s="15"/>
+      <c r="X22" s="15"/>
+      <c r="Y22" s="15"/>
+      <c r="Z22" s="15"/>
+      <c r="AA22" s="15"/>
+      <c r="AB22" s="15"/>
+      <c r="AC22" s="15"/>
+      <c r="AD22" s="15"/>
+      <c r="AE22" s="15"/>
+      <c r="AF22" s="15"/>
+      <c r="AG22" s="15"/>
+      <c r="AH22" s="15"/>
       <c r="AI22" s="2"/>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" ht="30" customHeight="1" spans="1:35">
       <c r="A23" s="1"/>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="29"/>
-      <c r="L23" s="29"/>
-      <c r="M23" s="29"/>
-      <c r="N23" s="29"/>
-      <c r="O23" s="29"/>
-      <c r="P23" s="29"/>
-      <c r="Q23" s="29"/>
-      <c r="R23" s="29"/>
-      <c r="S23" s="29"/>
-      <c r="T23" s="29"/>
-      <c r="U23" s="29"/>
-      <c r="V23" s="29"/>
-      <c r="W23" s="29"/>
-      <c r="X23" s="29"/>
-      <c r="Y23" s="29"/>
-      <c r="Z23" s="29"/>
-      <c r="AA23" s="29"/>
-      <c r="AB23" s="29"/>
-      <c r="AC23" s="29"/>
-      <c r="AD23" s="29"/>
-      <c r="AE23" s="29"/>
-      <c r="AF23" s="29"/>
-      <c r="AG23" s="29"/>
-      <c r="AH23" s="29"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="16"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="16"/>
+      <c r="T23" s="16"/>
+      <c r="U23" s="16"/>
+      <c r="V23" s="16"/>
+      <c r="W23" s="16"/>
+      <c r="X23" s="16"/>
+      <c r="Y23" s="16"/>
+      <c r="Z23" s="16"/>
+      <c r="AA23" s="16"/>
+      <c r="AB23" s="16"/>
+      <c r="AC23" s="16"/>
+      <c r="AD23" s="16"/>
+      <c r="AE23" s="16"/>
+      <c r="AF23" s="16"/>
+      <c r="AG23" s="16"/>
+      <c r="AH23" s="16"/>
       <c r="AI23" s="2"/>
     </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" ht="30" customHeight="1" spans="1:35">
       <c r="A24" s="1"/>
       <c r="B24" s="10" t="s">
         <v>16</v>
@@ -3308,40 +4133,40 @@
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="30"/>
-      <c r="K24" s="30"/>
-      <c r="L24" s="30"/>
-      <c r="M24" s="30"/>
-      <c r="N24" s="30"/>
-      <c r="O24" s="30"/>
-      <c r="P24" s="30"/>
-      <c r="Q24" s="30"/>
-      <c r="R24" s="30"/>
-      <c r="S24" s="30"/>
-      <c r="T24" s="30"/>
-      <c r="U24" s="30"/>
-      <c r="V24" s="30"/>
-      <c r="W24" s="30"/>
-      <c r="X24" s="30"/>
-      <c r="Y24" s="30"/>
-      <c r="Z24" s="30"/>
-      <c r="AA24" s="30"/>
-      <c r="AB24" s="30"/>
-      <c r="AC24" s="31" t="s">
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="17"/>
+      <c r="U24" s="17"/>
+      <c r="V24" s="17"/>
+      <c r="W24" s="17"/>
+      <c r="X24" s="17"/>
+      <c r="Y24" s="17"/>
+      <c r="Z24" s="17"/>
+      <c r="AA24" s="17"/>
+      <c r="AB24" s="17"/>
+      <c r="AC24" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="AD24" s="31"/>
-      <c r="AE24" s="31"/>
-      <c r="AF24" s="31"/>
-      <c r="AG24" s="31"/>
-      <c r="AH24" s="31"/>
+      <c r="AD24" s="18"/>
+      <c r="AE24" s="18"/>
+      <c r="AF24" s="18"/>
+      <c r="AG24" s="18"/>
+      <c r="AH24" s="18"/>
       <c r="AI24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" ht="30" customHeight="1" spans="1:35">
       <c r="A25" s="1"/>
       <c r="B25" s="10" t="s">
         <v>10</v>
@@ -3349,40 +4174,40 @@
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="30"/>
-      <c r="K25" s="30"/>
-      <c r="L25" s="30"/>
-      <c r="M25" s="30"/>
-      <c r="N25" s="30"/>
-      <c r="O25" s="30"/>
-      <c r="P25" s="30"/>
-      <c r="Q25" s="30"/>
-      <c r="R25" s="30"/>
-      <c r="S25" s="30"/>
-      <c r="T25" s="30"/>
-      <c r="U25" s="30"/>
-      <c r="V25" s="30"/>
-      <c r="W25" s="30"/>
-      <c r="X25" s="30"/>
-      <c r="Y25" s="30"/>
-      <c r="Z25" s="30"/>
-      <c r="AA25" s="30"/>
-      <c r="AB25" s="30"/>
-      <c r="AC25" s="31" t="s">
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="17"/>
+      <c r="N25" s="17"/>
+      <c r="O25" s="17"/>
+      <c r="P25" s="17"/>
+      <c r="Q25" s="17"/>
+      <c r="R25" s="17"/>
+      <c r="S25" s="17"/>
+      <c r="T25" s="17"/>
+      <c r="U25" s="17"/>
+      <c r="V25" s="17"/>
+      <c r="W25" s="17"/>
+      <c r="X25" s="17"/>
+      <c r="Y25" s="17"/>
+      <c r="Z25" s="17"/>
+      <c r="AA25" s="17"/>
+      <c r="AB25" s="17"/>
+      <c r="AC25" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="AD25" s="31"/>
-      <c r="AE25" s="31"/>
-      <c r="AF25" s="31"/>
-      <c r="AG25" s="31"/>
-      <c r="AH25" s="31"/>
+      <c r="AD25" s="18"/>
+      <c r="AE25" s="18"/>
+      <c r="AF25" s="18"/>
+      <c r="AG25" s="18"/>
+      <c r="AH25" s="18"/>
       <c r="AI25" s="2"/>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" ht="30" customHeight="1" spans="1:35">
       <c r="A26" s="1"/>
       <c r="B26" s="10" t="s">
         <v>89</v>
@@ -3390,77 +4215,77 @@
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="30"/>
-      <c r="K26" s="30"/>
-      <c r="L26" s="30"/>
-      <c r="M26" s="30"/>
-      <c r="N26" s="30"/>
-      <c r="O26" s="30"/>
-      <c r="P26" s="30"/>
-      <c r="Q26" s="30"/>
-      <c r="R26" s="30"/>
-      <c r="S26" s="30"/>
-      <c r="T26" s="30"/>
-      <c r="U26" s="30"/>
-      <c r="V26" s="30"/>
-      <c r="W26" s="30"/>
-      <c r="X26" s="30"/>
-      <c r="Y26" s="30"/>
-      <c r="Z26" s="30"/>
-      <c r="AA26" s="30"/>
-      <c r="AB26" s="30"/>
-      <c r="AC26" s="31" t="s">
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="17"/>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="17"/>
+      <c r="R26" s="17"/>
+      <c r="S26" s="17"/>
+      <c r="T26" s="17"/>
+      <c r="U26" s="17"/>
+      <c r="V26" s="17"/>
+      <c r="W26" s="17"/>
+      <c r="X26" s="17"/>
+      <c r="Y26" s="17"/>
+      <c r="Z26" s="17"/>
+      <c r="AA26" s="17"/>
+      <c r="AB26" s="17"/>
+      <c r="AC26" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="AD26" s="31"/>
-      <c r="AE26" s="31"/>
-      <c r="AF26" s="31"/>
-      <c r="AG26" s="31"/>
-      <c r="AH26" s="31"/>
+      <c r="AD26" s="18"/>
+      <c r="AE26" s="18"/>
+      <c r="AF26" s="18"/>
+      <c r="AG26" s="18"/>
+      <c r="AH26" s="18"/>
       <c r="AI26" s="2"/>
     </row>
-    <row r="27" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" ht="3.75" customHeight="1" spans="1:35">
       <c r="A27" s="1"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="22"/>
-      <c r="Q27" s="22"/>
-      <c r="R27" s="22"/>
-      <c r="S27" s="22"/>
-      <c r="T27" s="22"/>
-      <c r="U27" s="22"/>
-      <c r="V27" s="22"/>
-      <c r="W27" s="22"/>
-      <c r="X27" s="22"/>
-      <c r="Y27" s="22"/>
-      <c r="Z27" s="22"/>
-      <c r="AA27" s="22"/>
-      <c r="AB27" s="22"/>
-      <c r="AC27" s="22"/>
-      <c r="AD27" s="22"/>
-      <c r="AE27" s="22"/>
-      <c r="AF27" s="22"/>
-      <c r="AG27" s="22"/>
-      <c r="AH27" s="22"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19"/>
+      <c r="N27" s="19"/>
+      <c r="O27" s="19"/>
+      <c r="P27" s="19"/>
+      <c r="Q27" s="19"/>
+      <c r="R27" s="19"/>
+      <c r="S27" s="19"/>
+      <c r="T27" s="19"/>
+      <c r="U27" s="19"/>
+      <c r="V27" s="19"/>
+      <c r="W27" s="19"/>
+      <c r="X27" s="19"/>
+      <c r="Y27" s="19"/>
+      <c r="Z27" s="19"/>
+      <c r="AA27" s="19"/>
+      <c r="AB27" s="19"/>
+      <c r="AC27" s="19"/>
+      <c r="AD27" s="19"/>
+      <c r="AE27" s="19"/>
+      <c r="AF27" s="19"/>
+      <c r="AG27" s="19"/>
+      <c r="AH27" s="19"/>
       <c r="AI27" s="2"/>
     </row>
-    <row r="28" customFormat="false" ht="409.5" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" ht="409.5" hidden="1" customHeight="1" spans="1:35">
       <c r="A28" s="1" t="s">
         <v>69</v>
       </c>
@@ -3497,14 +4322,11 @@
       <c r="AF28" s="1"/>
       <c r="AG28" s="1"/>
       <c r="AH28" s="1"/>
-      <c r="AI28" s="23"/>
+      <c r="AI28" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="90">
-    <mergeCell ref="A1:A27"/>
     <mergeCell ref="B1:AH1"/>
-    <mergeCell ref="AI1:AI27"/>
-    <mergeCell ref="B2:AH3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="F4:V4"/>
     <mergeCell ref="W4:Z4"/>
@@ -3540,7 +4362,6 @@
     <mergeCell ref="N10:U10"/>
     <mergeCell ref="V10:AE10"/>
     <mergeCell ref="AF10:AH10"/>
-    <mergeCell ref="B11:E14"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="L11:M11"/>
     <mergeCell ref="N11:U11"/>
@@ -3561,7 +4382,6 @@
     <mergeCell ref="N14:U14"/>
     <mergeCell ref="V14:AE14"/>
     <mergeCell ref="AF14:AH14"/>
-    <mergeCell ref="B15:E17"/>
     <mergeCell ref="F15:K15"/>
     <mergeCell ref="L15:M15"/>
     <mergeCell ref="N15:U15"/>
@@ -3578,7 +4398,6 @@
     <mergeCell ref="V17:AE17"/>
     <mergeCell ref="AF17:AH17"/>
     <mergeCell ref="B18:AH18"/>
-    <mergeCell ref="B19:AH22"/>
     <mergeCell ref="B23:AH23"/>
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="F24:AB24"/>
@@ -3591,13 +4410,16 @@
     <mergeCell ref="AC26:AH26"/>
     <mergeCell ref="B27:AH27"/>
     <mergeCell ref="A28:AH28"/>
+    <mergeCell ref="A1:A27"/>
+    <mergeCell ref="AI1:AI27"/>
+    <mergeCell ref="B2:AH3"/>
+    <mergeCell ref="B11:E14"/>
+    <mergeCell ref="B15:E17"/>
+    <mergeCell ref="B19:AH22"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0" top="0.590277777777778" bottom="0" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0" right="0" top="0.590277777777778" bottom="0" header="0.511805555555556" footer="0.511805555555556"/>
+  <pageSetup paperSize="9" scale="84" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>